<commit_message>
correct username of daschland (#133)
</commit_message>
<xml_diff>
--- a/data/daschland_ontology/json_header.xlsx
+++ b/data/daschland_ontology/json_header.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11028"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noemivillars-amberg/Documents/Customer_Projects/daschland-scripts/data/daschland_ontology/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noraammann/Documents/Cloned_GitHub/0854-daschland-scripts/data/daschland_ontology/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB7368E9-6262-904A-85F8-0577B2286B2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C4129C7-D4E9-944D-A70C-A359943867B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="92">
   <si>
     <t>username</t>
   </si>
@@ -326,6 +326,9 @@
   <si>
     <t>Admin</t>
   </si>
+  <si>
+    <t>daschlandAdmin</t>
+  </si>
 </sst>
 </file>
 
@@ -443,7 +446,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -495,9 +498,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -15274,22 +15274,22 @@
       </c>
     </row>
     <row r="6" spans="1:24" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="21" t="s">
-        <v>89</v>
+      <c r="A6" s="2" t="s">
+        <v>91</v>
       </c>
       <c r="B6" t="s">
         <v>88</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="D6" s="21" t="s">
+      <c r="D6" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="F6" s="21" t="s">
+      <c r="F6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="21" t="s">
+      <c r="G6" s="2" t="s">
         <v>26</v>
       </c>
     </row>

</xml_diff>